<commit_message>
Phase 8 work before the refactor!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974AA1AD-F39E-414D-A749-8FF649A5E01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793BB855-B3A5-423D-A895-D4A3C431BFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="411">
   <si>
     <t>Current</t>
   </si>
@@ -1266,6 +1266,9 @@
   </si>
   <si>
     <t>Caught UP</t>
+  </si>
+  <si>
+    <t>Interact Dragon</t>
   </si>
 </sst>
 </file>
@@ -1643,7 +1646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5853A869-EFC3-49CB-8DC6-87B1B6715E26}">
-  <dimension ref="A1:AD155"/>
+  <dimension ref="A1:AE155"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
@@ -1791,7 +1794,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1802,7 +1805,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1813,7 +1816,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1824,7 +1827,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -1835,7 +1838,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1846,7 +1849,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1854,7 +1857,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1862,7 +1865,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1953,8 +1956,11 @@
       <c r="AD24">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AE24">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -2043,7 +2049,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -2135,7 +2141,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2215,7 +2221,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -2271,7 +2277,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -2312,7 +2318,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -2362,7 +2368,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -2436,7 +2442,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -2526,6 +2532,9 @@
       </c>
       <c r="AD32" t="s">
         <v>341</v>
+      </c>
+      <c r="AE32" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>